<commit_message>
Ajustes no layout do Relatório
</commit_message>
<xml_diff>
--- a/relatorios/marco2.xlsx
+++ b/relatorios/marco2.xlsx
@@ -620,13 +620,13 @@
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="2"/>

</xml_diff>

<commit_message>
Ajustes no layout de botôes
</commit_message>
<xml_diff>
--- a/relatorios/marco2.xlsx
+++ b/relatorios/marco2.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
   <si>
     <t>Nº Cartão</t>
   </si>
@@ -44,37 +44,31 @@
     <t>4000 0000 0000 0001</t>
   </si>
   <si>
-    <t>Primeira compra de Gilberto</t>
+    <t>Segunda compra de Gilberto Si</t>
+  </si>
+  <si>
+    <t>BAIXA</t>
+  </si>
+  <si>
+    <t>4000 0000 0000 0004</t>
+  </si>
+  <si>
+    <t>Primeira compra de Juliano</t>
+  </si>
+  <si>
+    <t>ALTA</t>
+  </si>
+  <si>
+    <t>Venda Gilberto otimizado agora teste novos botoes</t>
+  </si>
+  <si>
+    <t>sxyzH</t>
+  </si>
+  <si>
+    <t>Gilberto testando novos botoes</t>
   </si>
   <si>
     <t>MEDIA</t>
-  </si>
-  <si>
-    <t>Segunda compra de Gilberto</t>
-  </si>
-  <si>
-    <t>BAIXA</t>
-  </si>
-  <si>
-    <t>4000 0000 0000 0002</t>
-  </si>
-  <si>
-    <t>Primeira compra de Fernanda</t>
-  </si>
-  <si>
-    <t>4000 0000 0000 0004</t>
-  </si>
-  <si>
-    <t>Primeira compra de Juliano</t>
-  </si>
-  <si>
-    <t>ALTA</t>
-  </si>
-  <si>
-    <t>Venda Gilberto otimizado agora</t>
-  </si>
-  <si>
-    <t>sxyzH</t>
   </si>
   <si>
     <t>Resumo por Cartão</t>
@@ -467,13 +461,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" style="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" style="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -499,10 +493,10 @@
         <v>5</v>
       </c>
       <c r="B2" s="8">
-        <v>568</v>
+        <v>65</v>
       </c>
       <c r="C2" s="11">
-        <v>46101.971736111111</v>
+        <v>46102.51421296296</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>6</v>
@@ -513,53 +507,53 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B3" s="8">
-        <v>65</v>
+        <v>58499</v>
       </c>
       <c r="C3" s="11">
-        <v>46102.51421296296</v>
+        <v>46104.578935185185</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B4" s="8">
-        <v>335</v>
+        <v>8745</v>
       </c>
       <c r="C4" s="11">
-        <v>46104.576516203706</v>
+        <v>46104.72583333333</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="8">
+        <v>235</v>
+      </c>
+      <c r="C5" s="11">
+        <v>46104.77925925926</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="8">
-        <v>58499</v>
-      </c>
-      <c r="C5" s="11">
-        <v>46104.578935185185</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -567,34 +561,24 @@
         <v>5</v>
       </c>
       <c r="B6" s="8">
-        <v>8745</v>
+        <v>890</v>
       </c>
       <c r="C6" s="11">
-        <v>46104.72583333333</v>
+        <v>46106.725532407407</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="8">
-        <v>235</v>
-      </c>
-      <c r="C7" s="11">
-        <v>46104.77925925926</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A7" s="4"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
@@ -604,72 +588,52 @@
       <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
+      <c r="A9" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="B9" s="8"/>
       <c r="C9" s="11"/>
       <c r="D9" s="2"/>
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="11"/>
       <c r="D10" s="2"/>
       <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>19</v>
+      <c r="A11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="8">
+        <v>9700</v>
+      </c>
+      <c r="C11" s="11">
+        <v>3</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B12" s="8">
-        <v>9378</v>
+        <v>58734</v>
       </c>
       <c r="C12" s="11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="8">
-        <v>335</v>
-      </c>
-      <c r="C13" s="11">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="4"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="8">
-        <v>58734</v>
-      </c>
-      <c r="C14" s="11">
-        <v>2</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>